<commit_message>
Refine responsibility table per management decisions
Mark 60-qualified retention as a settled corporate decision, adopt 51
provisionally to move fast (validity checked in parallel), and confirm
the non-dedicated policy. Add a verification-principle callout: freeing
9 must reduce required headcount somewhere, or maintaining 60 is pure
added cost.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LS3dsYjEuJQEW6Yhcpbpzd
</commit_message>
<xml_diff>
--- a/CAZH_26W_役割分担・期限表.xlsx
+++ b/CAZH_26W_役割分担・期限表.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +61,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007A4B00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="005B6B7B"/>
       <sz val="9"/>
@@ -83,7 +89,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +123,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D68910"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="002E86C1"/>
       </patternFill>
     </fill>
@@ -126,7 +137,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -148,11 +159,25 @@
         <color rgb="00C9D6E4"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="00D68910"/>
+      </left>
+      <right style="medium">
+        <color rgb="00D68910"/>
+      </right>
+      <top style="medium">
+        <color rgb="00D68910"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00D68910"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -196,32 +221,38 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -589,7 +620,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -670,12 +701,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>本日の決定事項</t>
+          <t>決定事項（前提）</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>CA資格者60名を維持する方針を決定</t>
+          <t>CA資格者60名を維持する</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -685,27 +716,27 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>山田部長（CA/ZH・TR責任者）</t>
+          <t>会社（経営決定事項）</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>松石部長・岩佐専務</t>
+          <t>岩佐専務・松石部長・山田部長</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>2026/08/12</t>
+          <t>―（決定済）</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>本日決定</t>
+          <t>決定済み</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>58名ではなく60名。復便時にFMG担当便を減らさないため。</t>
+          <t>会社の経営決定事項。議論対象外。58名でなく60名（復便時にFMG担当便を減らさないため）。</t>
         </is>
       </c>
     </row>
@@ -715,42 +746,42 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>本日の決定事項</t>
+          <t>決定事項（前提）</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>CA/ZH実運用51名の妥当性を判断・決定</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>決定</t>
-        </is>
-      </c>
-      <c r="E5" s="15" t="inlineStr">
-        <is>
-          <t>山田部長（CA/ZH・TR責任者）</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>松石部長・遠藤麻美</t>
+          <t>CA/ZH実運用を51名として進める（妥当性検証は並行）</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>方針</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>松石部長（進行）／山田部長（検証）</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>遠藤麻美</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>2026/08/12</t>
+          <t>2026/08/12 進行</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>本日決定</t>
-        </is>
-      </c>
-      <c r="I5" s="16" t="inlineStr">
-        <is>
-          <t>51名案は松石部長提示。現行オペレーション成立可否を山田部長が判断。</t>
+          <t>暫定確定・検証中</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>妥当性検証は未了だが、早く走らせるため51名で進行。検証は並行して継続。</t>
         </is>
       </c>
     </row>
@@ -760,12 +791,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>本日の決定事項</t>
+          <t>決定事項（前提）</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>「60名全員をCA/ZH専任にはしない」方針を決定</t>
+          <t>60名全員をCA/ZH専任にはしない</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -775,22 +806,22 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>山田部長（CA/ZH・TR責任者）</t>
+          <t>旅客オペレーション本部（方針決定）</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>松石部長・岩佐専務</t>
+          <t>山田部長・松石部長</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>2026/08/12</t>
+          <t>―（決定済）</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>本日決定</t>
+          <t>決定済み</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
@@ -805,25 +836,25 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>本日の決定事項</t>
+          <t>決定事項（前提）</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>差分9名を他チーム兼務者として保有する方針を決定</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>決定</t>
-        </is>
-      </c>
-      <c r="E7" s="15" t="inlineStr">
+          <t>差分9名を他チーム兼務者として保有する</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>方針</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>山田部長（CA/ZH・TR責任者）</t>
         </is>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>松石部長・遠藤麻美</t>
         </is>
@@ -835,10 +866,10 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>本日決定</t>
-        </is>
-      </c>
-      <c r="I7" s="16" t="inlineStr">
+          <t>確定</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>60−51＝9名。余剰ではなく資格者60名の一員として保有。</t>
         </is>
@@ -855,22 +886,22 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>CA資格維持に必要な最低アサイン回数・条件を確認</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
+          <t>CA資格者60名を「採用ではなく維持」する具体策を確認</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>確認</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>山田部長（CA/ZH・TR責任者）</t>
+          <t>岡崎部長（成田空港事業部）</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>遠藤麻美（採用戦略部）</t>
+          <t>山田部長・遠藤麻美</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -885,7 +916,7 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>兼務設計の前提。何回/どの条件で資格維持できるか。</t>
+          <t>現有56名＋AM・VN等から4名を資格取得・兼務化。新規採用に頼らない。</t>
         </is>
       </c>
     </row>
@@ -900,22 +931,22 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>TR不足7名をCA資格者兼務で補完できるか確認</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
+          <t>CA資格維持に必要な最低アサイン回数・条件を確認</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>確認</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>山田部長（CA/ZH・TR責任者）</t>
         </is>
       </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>松石部長・遠藤麻美</t>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>遠藤麻美（採用戦略部）</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -928,9 +959,9 @@
           <t>未着手</t>
         </is>
       </c>
-      <c r="I9" s="16" t="inlineStr">
-        <is>
-          <t>9名のうち7名をTR兼務へ。新規採用7名を回避。</t>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>兼務設計の前提。何回/どの条件で資格維持できるか。</t>
         </is>
       </c>
     </row>
@@ -945,22 +976,22 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>CA資格者不足4名をAM・VN等から補完できるか確認</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="inlineStr">
+          <t>TR不足7名をCA資格者兼務で補完できるか確認</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>確認</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>岡崎部長（成田空港事業部）</t>
+          <t>山田部長（CA/ZH・TR責任者）</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>山田部長・遠藤麻美</t>
+          <t>松石部長・遠藤麻美</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -975,7 +1006,7 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>56→60名。AM・VN等は空港事業部所管。採用でなく既存在籍者の資格取得・兼務化で。</t>
+          <t>9名のうち7名をTR兼務へ。新規採用7名を回避。</t>
         </is>
       </c>
     </row>
@@ -993,17 +1024,17 @@
           <t>TR必要人数38名を26Wベースで再検証</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>確認</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>山田部長（CA/ZH・TR責任者）</t>
         </is>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>松石部長・遠藤麻美</t>
         </is>
@@ -1018,7 +1049,7 @@
           <t>未着手</t>
         </is>
       </c>
-      <c r="I11" s="16" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>38名という必要数そのものを26W基準で見直す。</t>
         </is>
@@ -1038,7 +1069,7 @@
           <t>受ける人数（兼務分）を他チームの必要人数へ組み込む設計</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>実行</t>
         </is>
@@ -1083,17 +1114,17 @@
           <t>各チーム(TR/AM/VN/VJ/RF/UL/5J)の必要・専任必須・兼務可能人数を整理</t>
         </is>
       </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>実行</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>松石部長（成田全体プラン）</t>
         </is>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>山田部長・岡崎部長・遠藤麻美</t>
         </is>
@@ -1108,7 +1139,7 @@
           <t>未着手</t>
         </is>
       </c>
-      <c r="I13" s="16" t="inlineStr">
+      <c r="I13" s="17" t="inlineStr">
         <is>
           <t>組み込み設計の基礎データ。CA/ZH・TR＝山田部長、空港事業部各チーム＝岡崎部長が提供。</t>
         </is>
@@ -1128,7 +1159,7 @@
           <t>成田全体の必要人数（283名）を再算定し削減効果を確認</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>実行</t>
         </is>
@@ -1155,211 +1186,219 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>283名からどれだけ減らせるか。60名維持と原価抑制の両立を検証。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>凡例：種別＝決定（当日確定）／確認（可否・条件の確認）／実行（設計・算定作業）　｜　黄色＝期限・ステータスの入力欄（確定後に更新）　｜　RACIのR＝Responsible（主担当・遂行責任者）、関係者＝C/I（相談・共有先）</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
+          <t>★9名を兼務に回した分、他チーム(TR等)の必要人数が減っているはず。283が減らなければ60名維持は純コスト増。数字で確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>★検証の原則：　CA/ZH実運用を60→51に下げ、余った9名を兼務へ回す。その分、TR等どこかの必要人数が減っていなければ論理破綻＝60名維持は純粋な原価増になる。「9名を落とした分、必要人数が減る」ことを成田全体（283名）の再算定で必ず数字で示す。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>凡例：種別＝決定（確定済・経営/方針決定）／方針（暫定確定して進行）／確認（可否・条件の確認）／実行（設計・算定作業）　｜　黄色＝期限・ステータスの入力欄（確定後に更新）　｜　RACIのR＝Responsible（主担当・遂行責任者）、関係者＝C/I（相談・共有先）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>体制（登場者）</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>氏名</t>
         </is>
       </c>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>所属</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D21" s="23" t="inlineStr">
         <is>
           <t>役割・立場</t>
         </is>
       </c>
-      <c r="G19" s="21" t="inlineStr">
+      <c r="G21" s="23" t="inlineStr">
         <is>
           <t>本表での位置づけ</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>岩佐専務</t>
-        </is>
-      </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>旅客オペレーション本部・本部長</t>
-        </is>
-      </c>
-      <c r="C20" s="23" t="n"/>
-      <c r="D20" s="22" t="inlineStr">
-        <is>
-          <t>本部全体の統括</t>
-        </is>
-      </c>
-      <c r="E20" s="23" t="n"/>
-      <c r="F20" s="23" t="n"/>
-      <c r="G20" s="9" t="inlineStr">
-        <is>
-          <t>承認（Accountable）</t>
-        </is>
-      </c>
-      <c r="H20" s="23" t="n"/>
-      <c r="I20" s="23" t="n"/>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>松石部長</t>
-        </is>
-      </c>
-      <c r="B21" s="24" t="inlineStr">
-        <is>
-          <t>成田空港事業部・本部長付部長</t>
-        </is>
-      </c>
-      <c r="C21" s="25" t="n"/>
-      <c r="D21" s="24" t="inlineStr">
-        <is>
-          <t>成田全体の人員プラン立案</t>
-        </is>
-      </c>
-      <c r="E21" s="25" t="n"/>
-      <c r="F21" s="25" t="n"/>
-      <c r="G21" s="16" t="inlineStr">
-        <is>
-          <t>R：組み込み設計／全体再算定</t>
-        </is>
-      </c>
-      <c r="H21" s="25" t="n"/>
-      <c r="I21" s="25" t="n"/>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>岡崎部長</t>
-        </is>
-      </c>
-      <c r="B22" s="22" t="inlineStr">
-        <is>
-          <t>成田空港事業部・担当部長</t>
-        </is>
-      </c>
-      <c r="C22" s="23" t="n"/>
-      <c r="D22" s="22" t="inlineStr">
-        <is>
-          <t>空港事業部各チーム（AM/VN/VJ/5J/RF/UL）所管</t>
-        </is>
-      </c>
-      <c r="E22" s="23" t="n"/>
-      <c r="F22" s="23" t="n"/>
+          <t>岩佐専務</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>旅客オペレーション本部・本部長</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="n"/>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>本部全体の統括</t>
+        </is>
+      </c>
+      <c r="E22" s="25" t="n"/>
+      <c r="F22" s="25" t="n"/>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>R：AM・VN等からの補完確認</t>
-        </is>
-      </c>
-      <c r="H22" s="23" t="n"/>
-      <c r="I22" s="23" t="n"/>
+          <t>承認（Accountable）</t>
+        </is>
+      </c>
+      <c r="H22" s="25" t="n"/>
+      <c r="I22" s="25" t="n"/>
     </row>
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>山田部長</t>
-        </is>
-      </c>
-      <c r="B23" s="24" t="inlineStr">
-        <is>
-          <t>成田ANA事業部・部長</t>
-        </is>
-      </c>
-      <c r="C23" s="25" t="n"/>
-      <c r="D23" s="24" t="inlineStr">
-        <is>
-          <t>CA/ZH・TR の責任者</t>
-        </is>
-      </c>
-      <c r="E23" s="25" t="n"/>
-      <c r="F23" s="25" t="n"/>
-      <c r="G23" s="16" t="inlineStr">
-        <is>
-          <t>R：CA/ZH・TR関連の決定/確認</t>
-        </is>
-      </c>
-      <c r="H23" s="25" t="n"/>
-      <c r="I23" s="25" t="n"/>
+          <t>松石部長</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>成田空港事業部・本部長付部長</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="n"/>
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>成田全体の人員プラン立案</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="n"/>
+      <c r="F23" s="27" t="n"/>
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>R：組み込み設計／全体再算定</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n"/>
+      <c r="I23" s="27" t="n"/>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t>岡崎部長</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>成田空港事業部・担当部長</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>空港事業部各チーム（AM/VN/VJ/5J/RF/UL）所管</t>
+        </is>
+      </c>
+      <c r="E24" s="25" t="n"/>
+      <c r="F24" s="25" t="n"/>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>R：AM・VN等からの補完確認</t>
+        </is>
+      </c>
+      <c r="H24" s="25" t="n"/>
+      <c r="I24" s="25" t="n"/>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>山田部長</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>成田ANA事業部・部長</t>
+        </is>
+      </c>
+      <c r="C25" s="27" t="n"/>
+      <c r="D25" s="26" t="inlineStr">
+        <is>
+          <t>CA/ZH・TR の責任者</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="n"/>
+      <c r="F25" s="27" t="n"/>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>R：CA/ZH・TR関連の決定/確認</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n"/>
+      <c r="I25" s="27" t="n"/>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>遠藤麻美</t>
         </is>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B26" s="24" t="inlineStr">
         <is>
           <t>採用戦略部</t>
         </is>
       </c>
-      <c r="C24" s="23" t="n"/>
-      <c r="D24" s="22" t="inlineStr">
+      <c r="C26" s="25" t="n"/>
+      <c r="D26" s="24" t="inlineStr">
         <is>
           <t>資料作成・事務局</t>
         </is>
       </c>
-      <c r="E24" s="23" t="n"/>
-      <c r="F24" s="23" t="n"/>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="E26" s="25" t="n"/>
+      <c r="F26" s="25" t="n"/>
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>C/I：全体調整・論点整理</t>
         </is>
       </c>
-      <c r="H24" s="23" t="n"/>
-      <c r="I24" s="23" t="n"/>
+      <c r="H26" s="25" t="n"/>
+      <c r="I26" s="25" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="29">
     <mergeCell ref="A22"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="A20"/>
+    <mergeCell ref="B25:C25"/>
     <mergeCell ref="A18:I18"/>
     <mergeCell ref="B22:C22"/>
-    <mergeCell ref="A23"/>
-    <mergeCell ref="A19"/>
     <mergeCell ref="G24:I24"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="A24"/>
-    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="A20:I20"/>
     <mergeCell ref="D24:F24"/>
+    <mergeCell ref="G25:I25"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="G22:I22"/>
-    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="A25"/>
+    <mergeCell ref="D26:F26"/>
     <mergeCell ref="G21:I21"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D19:F19"/>
     <mergeCell ref="B24:C24"/>
+    <mergeCell ref="A26"/>
     <mergeCell ref="A21"/>
-    <mergeCell ref="B20:C20"/>
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="G23:I23"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="D21:F21"/>
-    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>